<commit_message>
feat(gcard): add versioned cross-version comparison metrics
Generate 6 CSV files comparing model_score vs gcard_v2/v4/v5/v6:
- intent/zc segment matrices (distribution, FTR rate, amount risk)
- decile lift bins with score boundaries per version
- monthly segment OOT-OOS metrics by version
- score bin PSI stability by version

Validation: pytest 16 passed, jm project validate ok, jm report regenerated.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/projects/2026-05-fujie-gcard-v1/runs/2026-06-imported-gcard-main-lgbm/reports/model_report.xlsx
+++ b/projects/2026-05-fujie-gcard-v1/runs/2026-06-imported-gcard-main-lgbm/reports/model_report.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="模型描述" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="重要变量" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="变量筛选过程和模型参数" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="模型效果-每月效果" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="模型效果-模型sloping" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="模型效果-意愿交叉风险（DEV-OOS）" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="模型稳定性" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="模型描述" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="重要变量" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="变量筛选过程和模型参数" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="模型效果-每月效果" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="模型效果-模型sloping" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="模型效果-意愿交叉风险（DEV-OOS）" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="模型稳定性" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1324,7 +1324,7 @@
         </is>
       </c>
       <c r="B5" s="8" t="n">
-        <v>1820451.86158979</v>
+        <v>1820451.861589789</v>
       </c>
       <c r="C5" s="6" t="n">
         <v>340</v>
@@ -1534,7 +1534,7 @@
         </is>
       </c>
       <c r="B12" s="8" t="n">
-        <v>200764.3632984162</v>
+        <v>200764.3632984161</v>
       </c>
       <c r="C12" s="6" t="n">
         <v>602</v>
@@ -1982,7 +1982,7 @@
         </is>
       </c>
       <c r="B29" s="8" t="n">
-        <v>1820451.86158979</v>
+        <v>1820451.861589789</v>
       </c>
       <c r="C29" s="6" t="n">
         <v>340</v>
@@ -2192,7 +2192,7 @@
         </is>
       </c>
       <c r="B36" s="8" t="n">
-        <v>200764.3632984162</v>
+        <v>200764.3632984161</v>
       </c>
       <c r="C36" s="6" t="n">
         <v>602</v>
@@ -2972,7 +2972,7 @@
         </is>
       </c>
       <c r="B62" s="8" t="n">
-        <v>18557.33082413674</v>
+        <v>18557.33082413673</v>
       </c>
       <c r="C62" s="6" t="n">
         <v>289</v>
@@ -3962,7 +3962,7 @@
         </is>
       </c>
       <c r="B95" s="8" t="n">
-        <v>6598.728333882987</v>
+        <v>6598.728333882988</v>
       </c>
       <c r="C95" s="6" t="n">
         <v>337</v>

</xml_diff>